<commit_message>
xlsx: the case books of every set (26,098 cases in 79 books) saved by Excel and read back: every case computes as in the book sent but one LET Excel rewrites past the engine's 255-argument limit, and the values Excel stored equal its answers but one it does not repeat; an empty text result as Excel writes it (<v/>); empty text in the round trip
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/excel/xlsx/roundtrip/formulas-values.xlsx
+++ b/test/excel/xlsx/roundtrip/formulas-values.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Library/Containers/com.microsoft.Excel/Data/tmp/fxlsx-71511/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Library/Containers/com.microsoft.Excel/Data/tmp/fxlsx-96170/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BCE9047-FC83-374C-B2E8-08CB3912C228}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1AD161C5-FDCD-794F-AD62-0BCF9E5B81E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>x</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t>div</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -431,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -583,6 +586,16 @@
     <row r="26" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C26">
         <v>23</v>
+      </c>
+    </row>
+    <row r="27" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C27" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C28" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
xlsx through Excel: the round trip's nine new books and four changed ones, Excel 16.113 en-US and ru-RU; every file opens, hidden lines, the filter mode (on the sheet and on a table), the 1904 date system and iterative calculation come back as written, and Excel's values equal the 54 predicted cells; Excel saves built-in money, accounting and East Asian formats otherwise and escapes literal characters (known), and hides a row of height 0, which the engine counts; the writer always writes calcPr, as Excel otherwise keeps iteration on from the book opened before
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/excel/xlsx/roundtrip/formulas-values.xlsx
+++ b/test/excel/xlsx/roundtrip/formulas-values.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Library/Containers/com.microsoft.Excel/Data/tmp/fxlsx-96170/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Library/Containers/com.microsoft.Excel/Data/tmp/fxlsx-67743/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1AD161C5-FDCD-794F-AD62-0BCF9E5B81E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8D12925D-F961-0C48-8822-31119EF72211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>